<commit_message>
update data package at: 2026-08-27T12:53:16
</commit_message>
<xml_diff>
--- a/data/BASE_QDD_INVESTIMENTO.xlsx
+++ b/data/BASE_QDD_INVESTIMENTO.xlsx
@@ -588,7 +588,7 @@
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>4610</t>
+          <t>4610 - IMOBILIZAÇÕES</t>
         </is>
       </c>
       <c r="R2" t="n">
@@ -669,7 +669,7 @@
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>4610</t>
+          <t>4610 - IMOBILIZAÇÕES</t>
         </is>
       </c>
       <c r="R3" t="n">
@@ -750,7 +750,7 @@
       </c>
       <c r="Q4" t="inlineStr">
         <is>
-          <t>4610</t>
+          <t>4610 - IMOBILIZAÇÕES</t>
         </is>
       </c>
       <c r="R4" t="n">
@@ -831,7 +831,7 @@
       </c>
       <c r="Q5" t="inlineStr">
         <is>
-          <t>4610</t>
+          <t>4610 - IMOBILIZAÇÕES</t>
         </is>
       </c>
       <c r="R5" t="n">
@@ -912,7 +912,7 @@
       </c>
       <c r="Q6" t="inlineStr">
         <is>
-          <t>4610</t>
+          <t>4610 - IMOBILIZAÇÕES</t>
         </is>
       </c>
       <c r="R6" t="n">
@@ -993,7 +993,7 @@
       </c>
       <c r="Q7" t="inlineStr">
         <is>
-          <t>4610</t>
+          <t>4610 - IMOBILIZAÇÕES</t>
         </is>
       </c>
       <c r="R7" t="n">
@@ -1074,7 +1074,7 @@
       </c>
       <c r="Q8" t="inlineStr">
         <is>
-          <t>4610</t>
+          <t>4610 - IMOBILIZAÇÕES</t>
         </is>
       </c>
       <c r="R8" t="n">
@@ -1155,7 +1155,7 @@
       </c>
       <c r="Q9" t="inlineStr">
         <is>
-          <t>4610</t>
+          <t>4610 - IMOBILIZAÇÕES</t>
         </is>
       </c>
       <c r="R9" t="n">
@@ -1236,7 +1236,7 @@
       </c>
       <c r="Q10" t="inlineStr">
         <is>
-          <t>4810</t>
+          <t>4810 - OUTRAS APLICAÇÕES</t>
         </is>
       </c>
       <c r="R10" t="n">
@@ -1317,7 +1317,7 @@
       </c>
       <c r="Q11" t="inlineStr">
         <is>
-          <t>4510</t>
+          <t>4510 - PARTICIPAÇÃO SOCIETÁRIA</t>
         </is>
       </c>
       <c r="R11" t="n">
@@ -1398,7 +1398,7 @@
       </c>
       <c r="Q12" t="inlineStr">
         <is>
-          <t>4510</t>
+          <t>4510 - PARTICIPAÇÃO SOCIETÁRIA</t>
         </is>
       </c>
       <c r="R12" t="n">
@@ -1479,7 +1479,7 @@
       </c>
       <c r="Q13" t="inlineStr">
         <is>
-          <t>4810</t>
+          <t>4810 - OUTRAS APLICAÇÕES</t>
         </is>
       </c>
       <c r="R13" t="n">
@@ -1560,7 +1560,7 @@
       </c>
       <c r="Q14" t="inlineStr">
         <is>
-          <t>4810</t>
+          <t>4810 - OUTRAS APLICAÇÕES</t>
         </is>
       </c>
       <c r="R14" t="n">
@@ -1641,7 +1641,7 @@
       </c>
       <c r="Q15" t="inlineStr">
         <is>
-          <t>4810</t>
+          <t>4810 - OUTRAS APLICAÇÕES</t>
         </is>
       </c>
       <c r="R15" t="n">
@@ -1722,7 +1722,7 @@
       </c>
       <c r="Q16" t="inlineStr">
         <is>
-          <t>4810</t>
+          <t>4810 - OUTRAS APLICAÇÕES</t>
         </is>
       </c>
       <c r="R16" t="n">
@@ -1803,7 +1803,7 @@
       </c>
       <c r="Q17" t="inlineStr">
         <is>
-          <t>4810</t>
+          <t>4810 - OUTRAS APLICAÇÕES</t>
         </is>
       </c>
       <c r="R17" t="n">
@@ -1884,7 +1884,7 @@
       </c>
       <c r="Q18" t="inlineStr">
         <is>
-          <t>4810</t>
+          <t>4810 - OUTRAS APLICAÇÕES</t>
         </is>
       </c>
       <c r="R18" t="n">
@@ -1965,7 +1965,7 @@
       </c>
       <c r="Q19" t="inlineStr">
         <is>
-          <t>4610</t>
+          <t>4610 - IMOBILIZAÇÕES</t>
         </is>
       </c>
       <c r="R19" t="n">
@@ -2046,7 +2046,7 @@
       </c>
       <c r="Q20" t="inlineStr">
         <is>
-          <t>4610</t>
+          <t>4610 - IMOBILIZAÇÕES</t>
         </is>
       </c>
       <c r="R20" t="n">
@@ -2127,7 +2127,7 @@
       </c>
       <c r="Q21" t="inlineStr">
         <is>
-          <t>4610</t>
+          <t>4610 - IMOBILIZAÇÕES</t>
         </is>
       </c>
       <c r="R21" t="n">
@@ -2208,7 +2208,7 @@
       </c>
       <c r="Q22" t="inlineStr">
         <is>
-          <t>4810</t>
+          <t>4810 - OUTRAS APLICAÇÕES</t>
         </is>
       </c>
       <c r="R22" t="n">
@@ -2289,7 +2289,7 @@
       </c>
       <c r="Q23" t="inlineStr">
         <is>
-          <t>4810</t>
+          <t>4810 - OUTRAS APLICAÇÕES</t>
         </is>
       </c>
       <c r="R23" t="n">
@@ -2370,7 +2370,7 @@
       </c>
       <c r="Q24" t="inlineStr">
         <is>
-          <t>4610</t>
+          <t>4610 - IMOBILIZAÇÕES</t>
         </is>
       </c>
       <c r="R24" t="n">
@@ -2451,7 +2451,7 @@
       </c>
       <c r="Q25" t="inlineStr">
         <is>
-          <t>4610</t>
+          <t>4610 - IMOBILIZAÇÕES</t>
         </is>
       </c>
       <c r="R25" t="n">
@@ -2532,7 +2532,7 @@
       </c>
       <c r="Q26" t="inlineStr">
         <is>
-          <t>4610</t>
+          <t>4610 - IMOBILIZAÇÕES</t>
         </is>
       </c>
       <c r="R26" t="n">
@@ -2613,7 +2613,7 @@
       </c>
       <c r="Q27" t="inlineStr">
         <is>
-          <t>4610</t>
+          <t>4610 - IMOBILIZAÇÕES</t>
         </is>
       </c>
       <c r="R27" t="n">
@@ -2694,7 +2694,7 @@
       </c>
       <c r="Q28" t="inlineStr">
         <is>
-          <t>4610</t>
+          <t>4610 - IMOBILIZAÇÕES</t>
         </is>
       </c>
       <c r="R28" t="n">
@@ -2775,7 +2775,7 @@
       </c>
       <c r="Q29" t="inlineStr">
         <is>
-          <t>4610</t>
+          <t>4610 - IMOBILIZAÇÕES</t>
         </is>
       </c>
       <c r="R29" t="n">
@@ -2856,7 +2856,7 @@
       </c>
       <c r="Q30" t="inlineStr">
         <is>
-          <t>4610</t>
+          <t>4610 - IMOBILIZAÇÕES</t>
         </is>
       </c>
       <c r="R30" t="n">
@@ -2937,7 +2937,7 @@
       </c>
       <c r="Q31" t="inlineStr">
         <is>
-          <t>4610</t>
+          <t>4610 - IMOBILIZAÇÕES</t>
         </is>
       </c>
       <c r="R31" t="n">
@@ -3018,7 +3018,7 @@
       </c>
       <c r="Q32" t="inlineStr">
         <is>
-          <t>4610</t>
+          <t>4610 - IMOBILIZAÇÕES</t>
         </is>
       </c>
       <c r="R32" t="n">
@@ -3099,7 +3099,7 @@
       </c>
       <c r="Q33" t="inlineStr">
         <is>
-          <t>4610</t>
+          <t>4610 - IMOBILIZAÇÕES</t>
         </is>
       </c>
       <c r="R33" t="n">

</xml_diff>

<commit_message>
update data package at: 2026-09-09T07:42:59
</commit_message>
<xml_diff>
--- a/data/BASE_QDD_INVESTIMENTO.xlsx
+++ b/data/BASE_QDD_INVESTIMENTO.xlsx
@@ -588,7 +588,7 @@
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>IMOBILIZAÇÕES</t>
+          <t>4610 - IMOBILIZAÇÕES</t>
         </is>
       </c>
       <c r="R2" t="n">
@@ -673,7 +673,7 @@
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>IMOBILIZAÇÕES</t>
+          <t>4610 - IMOBILIZAÇÕES</t>
         </is>
       </c>
       <c r="R3" t="n">
@@ -758,7 +758,7 @@
       </c>
       <c r="Q4" t="inlineStr">
         <is>
-          <t>IMOBILIZAÇÕES</t>
+          <t>4610 - IMOBILIZAÇÕES</t>
         </is>
       </c>
       <c r="R4" t="n">
@@ -843,7 +843,7 @@
       </c>
       <c r="Q5" t="inlineStr">
         <is>
-          <t>IMOBILIZAÇÕES</t>
+          <t>4610 - IMOBILIZAÇÕES</t>
         </is>
       </c>
       <c r="R5" t="n">
@@ -928,7 +928,7 @@
       </c>
       <c r="Q6" t="inlineStr">
         <is>
-          <t>IMOBILIZAÇÕES</t>
+          <t>4610 - IMOBILIZAÇÕES</t>
         </is>
       </c>
       <c r="R6" t="n">
@@ -1013,7 +1013,7 @@
       </c>
       <c r="Q7" t="inlineStr">
         <is>
-          <t>IMOBILIZAÇÕES</t>
+          <t>4610 - IMOBILIZAÇÕES</t>
         </is>
       </c>
       <c r="R7" t="n">
@@ -1098,7 +1098,7 @@
       </c>
       <c r="Q8" t="inlineStr">
         <is>
-          <t>IMOBILIZAÇÕES</t>
+          <t>4610 - IMOBILIZAÇÕES</t>
         </is>
       </c>
       <c r="R8" t="n">
@@ -1183,7 +1183,7 @@
       </c>
       <c r="Q9" t="inlineStr">
         <is>
-          <t>IMOBILIZAÇÕES</t>
+          <t>4610 - IMOBILIZAÇÕES</t>
         </is>
       </c>
       <c r="R9" t="n">
@@ -1268,7 +1268,7 @@
       </c>
       <c r="Q10" t="inlineStr">
         <is>
-          <t>OUTRAS APLICAÇÕES</t>
+          <t>4810 - OUTRAS APLICAÇÕES</t>
         </is>
       </c>
       <c r="R10" t="n">
@@ -1353,7 +1353,7 @@
       </c>
       <c r="Q11" t="inlineStr">
         <is>
-          <t>PARTICIPAÇÃO SOCIETÁRIA</t>
+          <t>4510 - PARTICIPAÇÃO SOCIETÁRIA</t>
         </is>
       </c>
       <c r="R11" t="n">
@@ -1438,7 +1438,7 @@
       </c>
       <c r="Q12" t="inlineStr">
         <is>
-          <t>PARTICIPAÇÃO SOCIETÁRIA</t>
+          <t>4510 - PARTICIPAÇÃO SOCIETÁRIA</t>
         </is>
       </c>
       <c r="R12" t="n">
@@ -1523,7 +1523,7 @@
       </c>
       <c r="Q13" t="inlineStr">
         <is>
-          <t>OUTRAS APLICAÇÕES</t>
+          <t>4810 - OUTRAS APLICAÇÕES</t>
         </is>
       </c>
       <c r="R13" t="n">
@@ -1608,7 +1608,7 @@
       </c>
       <c r="Q14" t="inlineStr">
         <is>
-          <t>OUTRAS APLICAÇÕES</t>
+          <t>4810 - OUTRAS APLICAÇÕES</t>
         </is>
       </c>
       <c r="R14" t="n">
@@ -1693,7 +1693,7 @@
       </c>
       <c r="Q15" t="inlineStr">
         <is>
-          <t>OUTRAS APLICAÇÕES</t>
+          <t>4810 - OUTRAS APLICAÇÕES</t>
         </is>
       </c>
       <c r="R15" t="n">
@@ -1778,7 +1778,7 @@
       </c>
       <c r="Q16" t="inlineStr">
         <is>
-          <t>OUTRAS APLICAÇÕES</t>
+          <t>4810 - OUTRAS APLICAÇÕES</t>
         </is>
       </c>
       <c r="R16" t="n">
@@ -1863,7 +1863,7 @@
       </c>
       <c r="Q17" t="inlineStr">
         <is>
-          <t>OUTRAS APLICAÇÕES</t>
+          <t>4810 - OUTRAS APLICAÇÕES</t>
         </is>
       </c>
       <c r="R17" t="n">
@@ -1948,7 +1948,7 @@
       </c>
       <c r="Q18" t="inlineStr">
         <is>
-          <t>OUTRAS APLICAÇÕES</t>
+          <t>4810 - OUTRAS APLICAÇÕES</t>
         </is>
       </c>
       <c r="R18" t="n">
@@ -2033,7 +2033,7 @@
       </c>
       <c r="Q19" t="inlineStr">
         <is>
-          <t>IMOBILIZAÇÕES</t>
+          <t>4610 - IMOBILIZAÇÕES</t>
         </is>
       </c>
       <c r="R19" t="n">
@@ -2118,7 +2118,7 @@
       </c>
       <c r="Q20" t="inlineStr">
         <is>
-          <t>PARTICIPAÇÃO SOCIETÁRIA</t>
+          <t>4510 - PARTICIPAÇÃO SOCIETÁRIA</t>
         </is>
       </c>
       <c r="R20" t="n">
@@ -2203,7 +2203,7 @@
       </c>
       <c r="Q21" t="inlineStr">
         <is>
-          <t>IMOBILIZAÇÕES</t>
+          <t>4610 - IMOBILIZAÇÕES</t>
         </is>
       </c>
       <c r="R21" t="n">
@@ -2288,7 +2288,7 @@
       </c>
       <c r="Q22" t="inlineStr">
         <is>
-          <t>IMOBILIZAÇÕES</t>
+          <t>4610 - IMOBILIZAÇÕES</t>
         </is>
       </c>
       <c r="R22" t="n">
@@ -2373,7 +2373,7 @@
       </c>
       <c r="Q23" t="inlineStr">
         <is>
-          <t>OUTRAS APLICAÇÕES</t>
+          <t>4810 - OUTRAS APLICAÇÕES</t>
         </is>
       </c>
       <c r="R23" t="n">
@@ -2458,7 +2458,7 @@
       </c>
       <c r="Q24" t="inlineStr">
         <is>
-          <t>OUTRAS APLICAÇÕES</t>
+          <t>4810 - OUTRAS APLICAÇÕES</t>
         </is>
       </c>
       <c r="R24" t="n">
@@ -2543,7 +2543,7 @@
       </c>
       <c r="Q25" t="inlineStr">
         <is>
-          <t>IMOBILIZAÇÕES</t>
+          <t>4610 - IMOBILIZAÇÕES</t>
         </is>
       </c>
       <c r="R25" t="n">
@@ -2628,7 +2628,7 @@
       </c>
       <c r="Q26" t="inlineStr">
         <is>
-          <t>IMOBILIZAÇÕES</t>
+          <t>4610 - IMOBILIZAÇÕES</t>
         </is>
       </c>
       <c r="R26" t="n">
@@ -2713,7 +2713,7 @@
       </c>
       <c r="Q27" t="inlineStr">
         <is>
-          <t>IMOBILIZAÇÕES</t>
+          <t>4610 - IMOBILIZAÇÕES</t>
         </is>
       </c>
       <c r="R27" t="n">
@@ -2798,7 +2798,7 @@
       </c>
       <c r="Q28" t="inlineStr">
         <is>
-          <t>IMOBILIZAÇÕES</t>
+          <t>4610 - IMOBILIZAÇÕES</t>
         </is>
       </c>
       <c r="R28" t="n">
@@ -2883,7 +2883,7 @@
       </c>
       <c r="Q29" t="inlineStr">
         <is>
-          <t>IMOBILIZAÇÕES</t>
+          <t>4610 - IMOBILIZAÇÕES</t>
         </is>
       </c>
       <c r="R29" t="n">
@@ -2968,7 +2968,7 @@
       </c>
       <c r="Q30" t="inlineStr">
         <is>
-          <t>IMOBILIZAÇÕES</t>
+          <t>4610 - IMOBILIZAÇÕES</t>
         </is>
       </c>
       <c r="R30" t="n">
@@ -3053,7 +3053,7 @@
       </c>
       <c r="Q31" t="inlineStr">
         <is>
-          <t>IMOBILIZAÇÕES</t>
+          <t>4610 - IMOBILIZAÇÕES</t>
         </is>
       </c>
       <c r="R31" t="n">
@@ -3138,7 +3138,7 @@
       </c>
       <c r="Q32" t="inlineStr">
         <is>
-          <t>IMOBILIZAÇÕES</t>
+          <t>4610 - IMOBILIZAÇÕES</t>
         </is>
       </c>
       <c r="R32" t="n">
@@ -3223,7 +3223,7 @@
       </c>
       <c r="Q33" t="inlineStr">
         <is>
-          <t>IMOBILIZAÇÕES</t>
+          <t>4610 - IMOBILIZAÇÕES</t>
         </is>
       </c>
       <c r="R33" t="n">
@@ -3308,7 +3308,7 @@
       </c>
       <c r="Q34" t="inlineStr">
         <is>
-          <t>IMOBILIZAÇÕES</t>
+          <t>4610 - IMOBILIZAÇÕES</t>
         </is>
       </c>
       <c r="R34" t="n">

</xml_diff>

<commit_message>
update data package at: 2026-09-10T07:12:14
</commit_message>
<xml_diff>
--- a/data/BASE_QDD_INVESTIMENTO.xlsx
+++ b/data/BASE_QDD_INVESTIMENTO.xlsx
@@ -916,7 +916,7 @@
         <v>3010</v>
       </c>
       <c r="N6" t="n">
-        <v>1</v>
+        <v>1000</v>
       </c>
       <c r="O6" t="n">
         <v>0</v>
@@ -2871,7 +2871,7 @@
         <v>3001</v>
       </c>
       <c r="N29" t="n">
-        <v>1</v>
+        <v>1000</v>
       </c>
       <c r="O29" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
update data package at: 2026-09-11T09:06:24
</commit_message>
<xml_diff>
--- a/data/BASE_QDD_INVESTIMENTO.xlsx
+++ b/data/BASE_QDD_INVESTIMENTO.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:W34"/>
+  <dimension ref="A1:W35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -882,48 +882,48 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>SECRETARIA DE ESTADO DE DESENVOLVIMENTO ECONÔMICO - CEMIG HOLDING</t>
+          <t>SECRETARIA DE ESTADO DE DESENVOLVIMENTO ECONÔMICO - COHAB</t>
         </is>
       </c>
       <c r="D6" t="n">
         <v>3</v>
       </c>
       <c r="E6" t="n">
-        <v>5121</v>
+        <v>5071</v>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>COMPANHIA ENERGÉTICA DE MINAS GERAIS - CEMIG HOLDING</t>
+          <t>COMPANHIA DE HABITAÇÃO DO ESTADO DE MINAS GERAIS - COHAB</t>
         </is>
       </c>
       <c r="G6" t="inlineStr"/>
       <c r="H6" t="n">
-        <v>25</v>
+        <v>16</v>
       </c>
       <c r="I6" t="n">
-        <v>752</v>
+        <v>122</v>
       </c>
       <c r="J6" t="n">
-        <v>35</v>
+        <v>705</v>
       </c>
       <c r="K6" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="L6" t="n">
         <v>10</v>
       </c>
       <c r="M6" t="n">
-        <v>3010</v>
+        <v>6010</v>
       </c>
       <c r="N6" t="n">
-        <v>1000</v>
+        <v>36608798</v>
       </c>
       <c r="O6" t="n">
         <v>0</v>
       </c>
       <c r="P6" t="inlineStr">
         <is>
-          <t xml:space="preserve"> INVESTIMENTOS EM PARTICIPAÇÕES SOCIETÁRIAS CEMIG HOLDING</t>
+          <t>MANUTENÇÃO E ADEQUAÇÃO DA INFRAESTRUTURA ADMINISTRATIVA - COHAB</t>
         </is>
       </c>
       <c r="Q6" t="inlineStr">
@@ -949,12 +949,12 @@
       </c>
       <c r="V6" t="inlineStr">
         <is>
-          <t xml:space="preserve"> INVESTIMENTOS EM PARTICIPAÇÕES SOCIETÁRIAS CEMIG HOLDING</t>
+          <t>MANUTENÇÃO E ADEQUAÇÃO DA INFRAESTRUTURA ADMINISTRATIVA - COHAB</t>
         </is>
       </c>
       <c r="W6" t="inlineStr">
         <is>
-          <t>INVESTIMENTOS CEMIG</t>
+          <t>APOIO ÀS POLÍTICAS PÚBLICAS</t>
         </is>
       </c>
     </row>
@@ -995,20 +995,20 @@
         <v>3</v>
       </c>
       <c r="L7" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="M7" t="n">
-        <v>3011</v>
+        <v>3010</v>
       </c>
       <c r="N7" t="n">
-        <v>5282465</v>
+        <v>1000</v>
       </c>
       <c r="O7" t="n">
         <v>0</v>
       </c>
       <c r="P7" t="inlineStr">
         <is>
-          <t xml:space="preserve"> MANUTENÇÃO DA INFRAESTRUTURA DA CEMIG HOLDING</t>
+          <t xml:space="preserve"> INVESTIMENTOS EM PARTICIPAÇÕES SOCIETÁRIAS CEMIG HOLDING</t>
         </is>
       </c>
       <c r="Q7" t="inlineStr">
@@ -1034,7 +1034,7 @@
       </c>
       <c r="V7" t="inlineStr">
         <is>
-          <t xml:space="preserve"> MANUTENÇÃO DA INFRAESTRUTURA DA CEMIG HOLDING</t>
+          <t xml:space="preserve"> INVESTIMENTOS EM PARTICIPAÇÕES SOCIETÁRIAS CEMIG HOLDING</t>
         </is>
       </c>
       <c r="W7" t="inlineStr">
@@ -1052,48 +1052,48 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>SECRETARIA DE ESTADO DE DESENVOLVIMENTO ECONÔMICO - INVEST MINAS</t>
+          <t>SECRETARIA DE ESTADO DE DESENVOLVIMENTO ECONÔMICO - CEMIG HOLDING</t>
         </is>
       </c>
       <c r="D8" t="n">
         <v>3</v>
       </c>
       <c r="E8" t="n">
-        <v>5131</v>
+        <v>5121</v>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>AGÊNCIA DE PROMOÇÃO DE INVESTIMENTOS DE MINAS GERAIS - INVEST MINAS</t>
+          <t>COMPANHIA ENERGÉTICA DE MINAS GERAIS - CEMIG HOLDING</t>
         </is>
       </c>
       <c r="G8" t="inlineStr"/>
       <c r="H8" t="n">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="I8" t="n">
-        <v>122</v>
+        <v>752</v>
       </c>
       <c r="J8" t="n">
-        <v>142</v>
+        <v>35</v>
       </c>
       <c r="K8" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="L8" t="n">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="M8" t="n">
-        <v>6008</v>
+        <v>3011</v>
       </c>
       <c r="N8" t="n">
-        <v>323000</v>
+        <v>5282465</v>
       </c>
       <c r="O8" t="n">
         <v>0</v>
       </c>
       <c r="P8" t="inlineStr">
         <is>
-          <t>MANUTENÇÃO DA INFRAESTRUTURA ADMINISTRATIVA E OPERACIONAL DA INVEST MINAS</t>
+          <t xml:space="preserve"> MANUTENÇÃO DA INFRAESTRUTURA DA CEMIG HOLDING</t>
         </is>
       </c>
       <c r="Q8" t="inlineStr">
@@ -1102,11 +1102,11 @@
         </is>
       </c>
       <c r="R8" t="n">
-        <v>4610</v>
+        <v>4614</v>
       </c>
       <c r="S8" t="inlineStr">
         <is>
-          <t>IMOBILIZAÇÕES</t>
+          <t>MÁQUINAS, APARELHOS E EQUIPAMENTOS</t>
         </is>
       </c>
       <c r="T8" t="n">
@@ -1119,12 +1119,12 @@
       </c>
       <c r="V8" t="inlineStr">
         <is>
-          <t>MANUTENÇÃO DA INFRAESTRUTURA ADMINISTRATIVA E OPERACIONAL DA INVEST MINAS</t>
+          <t xml:space="preserve"> MANUTENÇÃO DA INFRAESTRUTURA DA CEMIG HOLDING</t>
         </is>
       </c>
       <c r="W8" t="inlineStr">
         <is>
-          <t>MANUTENÇÃO DA INFRAESTRUTURA ADMINISTRATIVA E OPERACIONAL - INVEST MINAS</t>
+          <t>INVESTIMENTOS CEMIG</t>
         </is>
       </c>
     </row>
@@ -1133,52 +1133,52 @@
         <v>2027</v>
       </c>
       <c r="B9" t="n">
-        <v>1500</v>
+        <v>1220</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>SECRETARIA DE ESTADO DE PLANEJAMENTO E GESTÃO - PRODEMGE</t>
+          <t>SECRETARIA DE ESTADO DE DESENVOLVIMENTO ECONÔMICO - INVEST MINAS</t>
         </is>
       </c>
       <c r="D9" t="n">
         <v>3</v>
       </c>
       <c r="E9" t="n">
-        <v>5141</v>
+        <v>5131</v>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>COMPANHIA DE TECNOLOGIA DA INFORMAÇÃO DO ESTADO DE MINAS GERAIS - PRODEMGE</t>
+          <t>AGÊNCIA DE PROMOÇÃO DE INVESTIMENTOS DE MINAS GERAIS - INVEST MINAS</t>
         </is>
       </c>
       <c r="G9" t="inlineStr"/>
       <c r="H9" t="n">
-        <v>4</v>
+        <v>22</v>
       </c>
       <c r="I9" t="n">
-        <v>126</v>
+        <v>122</v>
       </c>
       <c r="J9" t="n">
-        <v>30</v>
+        <v>142</v>
       </c>
       <c r="K9" t="n">
         <v>6</v>
       </c>
       <c r="L9" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="M9" t="n">
-        <v>6006</v>
+        <v>6008</v>
       </c>
       <c r="N9" t="n">
-        <v>16317109</v>
+        <v>323000</v>
       </c>
       <c r="O9" t="n">
         <v>0</v>
       </c>
       <c r="P9" t="inlineStr">
         <is>
-          <t>MANUTENÇÃO DAS UNIDADES PREDIAIS</t>
+          <t>MANUTENÇÃO DA INFRAESTRUTURA ADMINISTRATIVA E OPERACIONAL DA INVEST MINAS</t>
         </is>
       </c>
       <c r="Q9" t="inlineStr">
@@ -1187,11 +1187,11 @@
         </is>
       </c>
       <c r="R9" t="n">
-        <v>4613</v>
+        <v>4610</v>
       </c>
       <c r="S9" t="inlineStr">
         <is>
-          <t>OBRAS E INSTALAÇÕES</t>
+          <t>IMOBILIZAÇÕES</t>
         </is>
       </c>
       <c r="T9" t="n">
@@ -1204,12 +1204,12 @@
       </c>
       <c r="V9" t="inlineStr">
         <is>
-          <t>MANUTENÇÃO DAS UNIDADES PREDIAIS</t>
+          <t>MANUTENÇÃO DA INFRAESTRUTURA ADMINISTRATIVA E OPERACIONAL DA INVEST MINAS</t>
         </is>
       </c>
       <c r="W9" t="inlineStr">
         <is>
-          <t>SOLUÇÕES EM TECNOLOGIA DA INFORMAÇÃO E COMUNICAÇÃO</t>
+          <t>MANUTENÇÃO DA INFRAESTRUTURA ADMINISTRATIVA E OPERACIONAL - INVEST MINAS</t>
         </is>
       </c>
     </row>
@@ -1247,36 +1247,36 @@
         <v>30</v>
       </c>
       <c r="K10" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="L10" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="M10" t="n">
-        <v>8001</v>
+        <v>6006</v>
       </c>
       <c r="N10" t="n">
-        <v>58031337</v>
+        <v>16317109</v>
       </c>
       <c r="O10" t="n">
         <v>0</v>
       </c>
       <c r="P10" t="inlineStr">
         <is>
-          <t>AQUISIÇÃO DE HARDWARES E SOFTWARES PARA PRESTAÇÃO DE SERVIÇOS EM TECNOLOGIA DA INFORMAÇÃO E COMUNICAÇÃO</t>
+          <t>MANUTENÇÃO DAS UNIDADES PREDIAIS</t>
         </is>
       </c>
       <c r="Q10" t="inlineStr">
         <is>
-          <t>4810 - OUTRAS APLICAÇÕES</t>
+          <t>4610 - IMOBILIZAÇÕES</t>
         </is>
       </c>
       <c r="R10" t="n">
-        <v>4817</v>
+        <v>4613</v>
       </c>
       <c r="S10" t="inlineStr">
         <is>
-          <t>EQUIPAMENTOS E SOFTWARE</t>
+          <t>OBRAS E INSTALAÇÕES</t>
         </is>
       </c>
       <c r="T10" t="n">
@@ -1289,7 +1289,7 @@
       </c>
       <c r="V10" t="inlineStr">
         <is>
-          <t>AQUISIÇÃO DE HARDWARES E SOFTWARES PARA PRESTAÇÃO DE SERVIÇOS EM TECNOLOGIA DA INFORMAÇÃO E COMUNICAÇÃO</t>
+          <t>MANUTENÇÃO DAS UNIDADES PREDIAIS</t>
         </is>
       </c>
       <c r="W10" t="inlineStr">
@@ -1303,22 +1303,22 @@
         <v>2027</v>
       </c>
       <c r="B11" t="n">
-        <v>1220</v>
+        <v>1500</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>SECRETARIA DE ESTADO DE DESENVOLVIMENTO ECONÔMICO - MGI</t>
+          <t>SECRETARIA DE ESTADO DE PLANEJAMENTO E GESTÃO - PRODEMGE</t>
         </is>
       </c>
       <c r="D11" t="n">
         <v>3</v>
       </c>
       <c r="E11" t="n">
-        <v>5191</v>
+        <v>5141</v>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>MINAS GERAIS PARTICIPAÇÕES S.A - MGI</t>
+          <t>COMPANHIA DE TECNOLOGIA DA INFORMAÇÃO DO ESTADO DE MINAS GERAIS - PRODEMGE</t>
         </is>
       </c>
       <c r="G11" t="inlineStr"/>
@@ -1326,60 +1326,60 @@
         <v>4</v>
       </c>
       <c r="I11" t="n">
-        <v>123</v>
+        <v>126</v>
       </c>
       <c r="J11" t="n">
-        <v>13</v>
+        <v>30</v>
       </c>
       <c r="K11" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="L11" t="n">
         <v>1</v>
       </c>
       <c r="M11" t="n">
-        <v>6001</v>
+        <v>8001</v>
       </c>
       <c r="N11" t="n">
-        <v>1000</v>
+        <v>58031337</v>
       </c>
       <c r="O11" t="n">
         <v>0</v>
       </c>
       <c r="P11" t="inlineStr">
         <is>
-          <t>INVESTIMENTOS VIA PARTICIPAÇÃO SOCIETÁRIA</t>
+          <t>AQUISIÇÃO DE HARDWARES E SOFTWARES PARA PRESTAÇÃO DE SERVIÇOS EM TECNOLOGIA DA INFORMAÇÃO E COMUNICAÇÃO</t>
         </is>
       </c>
       <c r="Q11" t="inlineStr">
         <is>
-          <t>4510 - PARTICIPAÇÃO SOCIETÁRIA</t>
+          <t>4810 - OUTRAS APLICAÇÕES</t>
         </is>
       </c>
       <c r="R11" t="n">
-        <v>4511</v>
+        <v>4817</v>
       </c>
       <c r="S11" t="inlineStr">
         <is>
-          <t>SOCIEDADES CONTROLADAS</t>
+          <t>EQUIPAMENTOS E SOFTWARE</t>
         </is>
       </c>
       <c r="T11" t="n">
-        <v>11101</v>
+        <v>51000</v>
       </c>
       <c r="U11" t="inlineStr">
         <is>
-          <t>TESOURO ORDINÁRIO - APLICAÇÃO LIVRE</t>
+          <t>RECURSOS PRÓPRIOS</t>
         </is>
       </c>
       <c r="V11" t="inlineStr">
         <is>
-          <t>INVESTIMENTOS VIA PARTICIPAÇÃO SOCIETÁRIA</t>
+          <t>AQUISIÇÃO DE HARDWARES E SOFTWARES PARA PRESTAÇÃO DE SERVIÇOS EM TECNOLOGIA DA INFORMAÇÃO E COMUNICAÇÃO</t>
         </is>
       </c>
       <c r="W11" t="inlineStr">
         <is>
-          <t>APORTE DE CAPITAL E MANUTENÇÃO DA INFRAESTRUTURA DA MGI</t>
+          <t>SOLUÇÕES EM TECNOLOGIA DA INFORMAÇÃO E COMUNICAÇÃO</t>
         </is>
       </c>
     </row>
@@ -1450,11 +1450,11 @@
         </is>
       </c>
       <c r="T12" t="n">
-        <v>51000</v>
+        <v>11101</v>
       </c>
       <c r="U12" t="inlineStr">
         <is>
-          <t>RECURSOS PRÓPRIOS</t>
+          <t>TESOURO ORDINÁRIO - APLICAÇÃO LIVRE</t>
         </is>
       </c>
       <c r="V12" t="inlineStr">
@@ -1496,7 +1496,7 @@
         <v>4</v>
       </c>
       <c r="I13" t="n">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="J13" t="n">
         <v>13</v>
@@ -1505,33 +1505,33 @@
         <v>6</v>
       </c>
       <c r="L13" t="n">
-        <v>11</v>
+        <v>1</v>
       </c>
       <c r="M13" t="n">
-        <v>6011</v>
+        <v>6001</v>
       </c>
       <c r="N13" t="n">
-        <v>555000</v>
+        <v>1000</v>
       </c>
       <c r="O13" t="n">
         <v>0</v>
       </c>
       <c r="P13" t="inlineStr">
         <is>
-          <t>MANUTENÇÃO E ADEQUAÇÃO DA INFRAESTRUTURA DA MGI</t>
+          <t>INVESTIMENTOS VIA PARTICIPAÇÃO SOCIETÁRIA</t>
         </is>
       </c>
       <c r="Q13" t="inlineStr">
         <is>
-          <t>4810 - OUTRAS APLICAÇÕES</t>
+          <t>4510 - PARTICIPAÇÃO SOCIETÁRIA</t>
         </is>
       </c>
       <c r="R13" t="n">
-        <v>4817</v>
+        <v>4511</v>
       </c>
       <c r="S13" t="inlineStr">
         <is>
-          <t>EQUIPAMENTOS E SOFTWARE</t>
+          <t>SOCIEDADES CONTROLADAS</t>
         </is>
       </c>
       <c r="T13" t="n">
@@ -1544,7 +1544,7 @@
       </c>
       <c r="V13" t="inlineStr">
         <is>
-          <t>MANUTENÇÃO E ADEQUAÇÃO DA INFRAESTRUTURA DA MGI</t>
+          <t>INVESTIMENTOS VIA PARTICIPAÇÃO SOCIETÁRIA</t>
         </is>
       </c>
       <c r="W13" t="inlineStr">
@@ -1584,26 +1584,26 @@
         <v>122</v>
       </c>
       <c r="J14" t="n">
-        <v>119</v>
+        <v>13</v>
       </c>
       <c r="K14" t="n">
         <v>6</v>
       </c>
       <c r="L14" t="n">
-        <v>3</v>
+        <v>11</v>
       </c>
       <c r="M14" t="n">
-        <v>6003</v>
+        <v>6011</v>
       </c>
       <c r="N14" t="n">
-        <v>1000</v>
+        <v>555000</v>
       </c>
       <c r="O14" t="n">
         <v>0</v>
       </c>
       <c r="P14" t="inlineStr">
         <is>
-          <t>SUPORTE AO DESENVOLVIMENTO ESTADUAL</t>
+          <t>MANUTENÇÃO E ADEQUAÇÃO DA INFRAESTRUTURA DA MGI</t>
         </is>
       </c>
       <c r="Q14" t="inlineStr">
@@ -1612,29 +1612,29 @@
         </is>
       </c>
       <c r="R14" t="n">
-        <v>4819</v>
+        <v>4817</v>
       </c>
       <c r="S14" t="inlineStr">
         <is>
-          <t>OUTRAS APLICAÇÕES</t>
+          <t>EQUIPAMENTOS E SOFTWARE</t>
         </is>
       </c>
       <c r="T14" t="n">
-        <v>11101</v>
+        <v>51000</v>
       </c>
       <c r="U14" t="inlineStr">
         <is>
-          <t>TESOURO ORDINÁRIO - APLICAÇÃO LIVRE</t>
+          <t>RECURSOS PRÓPRIOS</t>
         </is>
       </c>
       <c r="V14" t="inlineStr">
         <is>
-          <t>SUPORTE AO DESENVOLVIMENTO ESTADUAL</t>
+          <t>MANUTENÇÃO E ADEQUAÇÃO DA INFRAESTRUTURA DA MGI</t>
         </is>
       </c>
       <c r="W14" t="inlineStr">
         <is>
-          <t>Apoio ao Desenvolvimento Municipal e à Coordenação das Transferências Estaduais de Recursos Financeiros</t>
+          <t>APORTE DE CAPITAL E MANUTENÇÃO DA INFRAESTRUTURA DA MGI</t>
         </is>
       </c>
     </row>
@@ -1681,7 +1681,7 @@
         <v>6003</v>
       </c>
       <c r="N15" t="n">
-        <v>664500</v>
+        <v>1000</v>
       </c>
       <c r="O15" t="n">
         <v>0</v>
@@ -1705,11 +1705,11 @@
         </is>
       </c>
       <c r="T15" t="n">
-        <v>51000</v>
+        <v>11101</v>
       </c>
       <c r="U15" t="inlineStr">
         <is>
-          <t>RECURSOS PRÓPRIOS</t>
+          <t>TESOURO ORDINÁRIO - APLICAÇÃO LIVRE</t>
         </is>
       </c>
       <c r="V15" t="inlineStr">
@@ -1732,48 +1732,48 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>SECRETARIA DE ESTADO DE DESENVOLVIMENTO ECONÔMICO - BDMG</t>
+          <t>SECRETARIA DE ESTADO DE DESENVOLVIMENTO ECONÔMICO - MGI</t>
         </is>
       </c>
       <c r="D16" t="n">
         <v>3</v>
       </c>
       <c r="E16" t="n">
-        <v>5201</v>
+        <v>5191</v>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>BANCO DE DESENVOLVIMENTO DE MINAS GERAIS S.A - BDMG</t>
+          <t>MINAS GERAIS PARTICIPAÇÕES S.A - MGI</t>
         </is>
       </c>
       <c r="G16" t="inlineStr"/>
       <c r="H16" t="n">
-        <v>23</v>
+        <v>4</v>
       </c>
       <c r="I16" t="n">
-        <v>694</v>
+        <v>122</v>
       </c>
       <c r="J16" t="n">
-        <v>14</v>
+        <v>119</v>
       </c>
       <c r="K16" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="L16" t="n">
         <v>3</v>
       </c>
       <c r="M16" t="n">
-        <v>8003</v>
+        <v>6003</v>
       </c>
       <c r="N16" t="n">
-        <v>260000000</v>
+        <v>664500</v>
       </c>
       <c r="O16" t="n">
         <v>0</v>
       </c>
       <c r="P16" t="inlineStr">
         <is>
-          <t>FINANCIAMENTO À DESCARBONIZAÇÃO E RESILIÊNCIA CLIMÁTICA ENTRE BDMG E BANCO INTERAMERICANO DE DESENVOLVIMENTO (BDMG PBR)</t>
+          <t>SUPORTE AO DESENVOLVIMENTO ESTADUAL</t>
         </is>
       </c>
       <c r="Q16" t="inlineStr">
@@ -1782,7 +1782,7 @@
         </is>
       </c>
       <c r="R16" t="n">
-        <v>4810</v>
+        <v>4819</v>
       </c>
       <c r="S16" t="inlineStr">
         <is>
@@ -1790,21 +1790,21 @@
         </is>
       </c>
       <c r="T16" t="n">
-        <v>12400</v>
+        <v>51000</v>
       </c>
       <c r="U16" t="inlineStr">
         <is>
-          <t>OUTRAS ENTIDADES - BDMG</t>
+          <t>RECURSOS PRÓPRIOS</t>
         </is>
       </c>
       <c r="V16" t="inlineStr">
         <is>
-          <t>FINANCIAMENTO À DESCARBONIZAÇÃO E RESILIÊNCIA CLIMÁTICA ENTRE BDMG E BANCO INTERAMERICANO DE DESENVOLVIMENTO (BDMG PBR)</t>
+          <t>SUPORTE AO DESENVOLVIMENTO ESTADUAL</t>
         </is>
       </c>
       <c r="W16" t="inlineStr">
         <is>
-          <t>FINANCIAMENTO À DESCARBONIZAÇÃO E RESILIÊNCIA CLIMÁTICA ENTRE BDMG E BANCO INTERAMERICANO DE DESENVOLVIMENTO (BDMG PBR)</t>
+          <t>Apoio ao Desenvolvimento Municipal e à Coordenação das Transferências Estaduais de Recursos Financeiros</t>
         </is>
       </c>
     </row>
@@ -1836,29 +1836,29 @@
         <v>23</v>
       </c>
       <c r="I17" t="n">
-        <v>122</v>
+        <v>694</v>
       </c>
       <c r="J17" t="n">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="K17" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="L17" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="M17" t="n">
-        <v>6004</v>
+        <v>8003</v>
       </c>
       <c r="N17" t="n">
-        <v>38941920</v>
+        <v>260000000</v>
       </c>
       <c r="O17" t="n">
         <v>0</v>
       </c>
       <c r="P17" t="inlineStr">
         <is>
-          <t>MANUTENÇÃO E ADEQUAÇÃO DA INFRA-ESTRUTURA ADMINISTRATIVA E OPERACIONAL DO BDMG</t>
+          <t>FINANCIAMENTO À DESCARBONIZAÇÃO E RESILIÊNCIA CLIMÁTICA ENTRE BDMG E BANCO INTERAMERICANO DE DESENVOLVIMENTO (BDMG PBR)</t>
         </is>
       </c>
       <c r="Q17" t="inlineStr">
@@ -1867,11 +1867,11 @@
         </is>
       </c>
       <c r="R17" t="n">
-        <v>4813</v>
+        <v>4810</v>
       </c>
       <c r="S17" t="inlineStr">
         <is>
-          <t>INTANGÍVEIS E OUTROS INVESTIMENTOS</t>
+          <t>OUTRAS APLICAÇÕES</t>
         </is>
       </c>
       <c r="T17" t="n">
@@ -1884,12 +1884,12 @@
       </c>
       <c r="V17" t="inlineStr">
         <is>
-          <t>MANUTENÇÃO E ADEQUAÇÃO DA INFRA-ESTRUTURA ADMINISTRATIVA E OPERACIONAL DO BDMG</t>
+          <t>FINANCIAMENTO À DESCARBONIZAÇÃO E RESILIÊNCIA CLIMÁTICA ENTRE BDMG E BANCO INTERAMERICANO DE DESENVOLVIMENTO (BDMG PBR)</t>
         </is>
       </c>
       <c r="W17" t="inlineStr">
         <is>
-          <t>INVESTIMENTO NA INFRAESTRUTURA ADMINISTRATIVA E OPERACIONAL  DO BDMG</t>
+          <t>FINANCIAMENTO À DESCARBONIZAÇÃO E RESILIÊNCIA CLIMÁTICA ENTRE BDMG E BANCO INTERAMERICANO DE DESENVOLVIMENTO (BDMG PBR)</t>
         </is>
       </c>
     </row>
@@ -1921,29 +1921,29 @@
         <v>23</v>
       </c>
       <c r="I18" t="n">
-        <v>694</v>
+        <v>122</v>
       </c>
       <c r="J18" t="n">
-        <v>107</v>
+        <v>17</v>
       </c>
       <c r="K18" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="L18" t="n">
         <v>4</v>
       </c>
       <c r="M18" t="n">
-        <v>8004</v>
+        <v>6004</v>
       </c>
       <c r="N18" t="n">
-        <v>825000000</v>
+        <v>38941920</v>
       </c>
       <c r="O18" t="n">
         <v>0</v>
       </c>
       <c r="P18" t="inlineStr">
         <is>
-          <t>FINANCIAMENTO À SUSTENTABILIDADE E ÀS MICRO E PEQUENAS EMPRESAS DO ESTADO DE MINAS GERAIS ENTRE BDMG E BANCO EUROPEU DE INVESTIMENTO (BDMG SUSTENTABILIDADE E MPE)</t>
+          <t>MANUTENÇÃO E ADEQUAÇÃO DA INFRA-ESTRUTURA ADMINISTRATIVA E OPERACIONAL DO BDMG</t>
         </is>
       </c>
       <c r="Q18" t="inlineStr">
@@ -1952,11 +1952,11 @@
         </is>
       </c>
       <c r="R18" t="n">
-        <v>4810</v>
+        <v>4813</v>
       </c>
       <c r="S18" t="inlineStr">
         <is>
-          <t>OUTRAS APLICAÇÕES</t>
+          <t>INTANGÍVEIS E OUTROS INVESTIMENTOS</t>
         </is>
       </c>
       <c r="T18" t="n">
@@ -1969,12 +1969,12 @@
       </c>
       <c r="V18" t="inlineStr">
         <is>
-          <t>FINANCIAMENTO À SUSTENTABILIDADE E ÀS MICRO E PEQUENAS EMPRESAS DO ESTADO DE MINAS GERAIS ENTRE BDMG E BANCO EUROPEU DE INVESTIMENTO (BDMG SUSTENTABILIDADE E MPE)</t>
+          <t>MANUTENÇÃO E ADEQUAÇÃO DA INFRA-ESTRUTURA ADMINISTRATIVA E OPERACIONAL DO BDMG</t>
         </is>
       </c>
       <c r="W18" t="inlineStr">
         <is>
-          <t xml:space="preserve">FINANCIAMENTO À SUSTENTABILIDADE E ÀS MICRO E PEQUENAS EMPRESAS DO ESTADO DE MINAS GERAIS ENTRE BDMG E BANCO EUROPEU DE </t>
+          <t>INVESTIMENTO NA INFRAESTRUTURA ADMINISTRATIVA E OPERACIONAL  DO BDMG</t>
         </is>
       </c>
     </row>
@@ -1987,79 +1987,79 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>SECRETARIA DE ESTADO DE DESENVOLVIMENTO ECONÔMICO - GASMIG</t>
+          <t>SECRETARIA DE ESTADO DE DESENVOLVIMENTO ECONÔMICO - BDMG</t>
         </is>
       </c>
       <c r="D19" t="n">
         <v>3</v>
       </c>
       <c r="E19" t="n">
-        <v>5251</v>
+        <v>5201</v>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>COMPANHIA DE GÁS DE MINAS GERAIS - GASMIG</t>
+          <t>BANCO DE DESENVOLVIMENTO DE MINAS GERAIS S.A - BDMG</t>
         </is>
       </c>
       <c r="G19" t="inlineStr"/>
       <c r="H19" t="n">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="I19" t="n">
-        <v>121</v>
+        <v>694</v>
       </c>
       <c r="J19" t="n">
-        <v>133</v>
+        <v>107</v>
       </c>
       <c r="K19" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="L19" t="n">
-        <v>18</v>
+        <v>4</v>
       </c>
       <c r="M19" t="n">
-        <v>3018</v>
+        <v>8004</v>
       </c>
       <c r="N19" t="n">
-        <v>457766318</v>
+        <v>825000000</v>
       </c>
       <c r="O19" t="n">
         <v>0</v>
       </c>
       <c r="P19" t="inlineStr">
         <is>
-          <t>GÁS COMPETITIVO- EXPANSÃO DA REDE DE GÁS NATURAL</t>
+          <t>FINANCIAMENTO À SUSTENTABILIDADE E ÀS MICRO E PEQUENAS EMPRESAS DO ESTADO DE MINAS GERAIS ENTRE BDMG E BANCO EUROPEU DE INVESTIMENTO (BDMG SUSTENTABILIDADE E MPE)</t>
         </is>
       </c>
       <c r="Q19" t="inlineStr">
         <is>
-          <t>4610 - IMOBILIZAÇÕES</t>
+          <t>4810 - OUTRAS APLICAÇÕES</t>
         </is>
       </c>
       <c r="R19" t="n">
-        <v>4613</v>
+        <v>4810</v>
       </c>
       <c r="S19" t="inlineStr">
         <is>
-          <t>OBRAS E INSTALAÇÕES</t>
+          <t>OUTRAS APLICAÇÕES</t>
         </is>
       </c>
       <c r="T19" t="n">
-        <v>51000</v>
+        <v>12400</v>
       </c>
       <c r="U19" t="inlineStr">
         <is>
-          <t>RECURSOS PRÓPRIOS</t>
+          <t>OUTRAS ENTIDADES - BDMG</t>
         </is>
       </c>
       <c r="V19" t="inlineStr">
         <is>
-          <t>GÁS COMPETITIVO- EXPANSÃO DA REDE DE GÁS NATURAL</t>
+          <t>FINANCIAMENTO À SUSTENTABILIDADE E ÀS MICRO E PEQUENAS EMPRESAS DO ESTADO DE MINAS GERAIS ENTRE BDMG E BANCO EUROPEU DE INVESTIMENTO (BDMG SUSTENTABILIDADE E MPE)</t>
         </is>
       </c>
       <c r="W19" t="inlineStr">
         <is>
-          <t>MINAS GERAÇÃO DE VALOR</t>
+          <t xml:space="preserve">FINANCIAMENTO À SUSTENTABILIDADE E ÀS MICRO E PEQUENAS EMPRESAS DO ESTADO DE MINAS GERAIS ENTRE BDMG E BANCO EUROPEU DE </t>
         </is>
       </c>
     </row>
@@ -2068,83 +2068,83 @@
         <v>2027</v>
       </c>
       <c r="B20" t="n">
-        <v>1300</v>
+        <v>1220</v>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>SECRETARIA DE ESTADO DE INFRAESTRUTURA, MOBILIDADE E PARCERIA - TREM METROPOLITANO</t>
+          <t>SECRETARIA DE ESTADO DE DESENVOLVIMENTO ECONÔMICO - GASMIG</t>
         </is>
       </c>
       <c r="D20" t="n">
         <v>3</v>
       </c>
       <c r="E20" t="n">
-        <v>5261</v>
+        <v>5251</v>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>TREM METROPOLITANO DE BELO HORIZONTE S.A - TREM METROPOLITANO</t>
+          <t>COMPANHIA DE GÁS DE MINAS GERAIS - GASMIG</t>
         </is>
       </c>
       <c r="G20" t="inlineStr"/>
       <c r="H20" t="n">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="I20" t="n">
-        <v>783</v>
+        <v>121</v>
       </c>
       <c r="J20" t="n">
-        <v>705</v>
+        <v>133</v>
       </c>
       <c r="K20" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="L20" t="n">
-        <v>11</v>
+        <v>18</v>
       </c>
       <c r="M20" t="n">
-        <v>8011</v>
+        <v>3018</v>
       </c>
       <c r="N20" t="n">
-        <v>1000</v>
+        <v>457766318</v>
       </c>
       <c r="O20" t="n">
         <v>0</v>
       </c>
       <c r="P20" t="inlineStr">
         <is>
-          <t>MANUTENÇÃO E ADEQUAÇÃO DA INFRA-ESTRUTURA ADMINISTRATIVA E OPERACIONAL - TRANSPORTES METROPOLITANOS</t>
+          <t>GÁS COMPETITIVO- EXPANSÃO DA REDE DE GÁS NATURAL</t>
         </is>
       </c>
       <c r="Q20" t="inlineStr">
         <is>
-          <t>4510 - PARTICIPAÇÃO SOCIETÁRIA</t>
+          <t>4610 - IMOBILIZAÇÕES</t>
         </is>
       </c>
       <c r="R20" t="n">
-        <v>4511</v>
+        <v>4613</v>
       </c>
       <c r="S20" t="inlineStr">
         <is>
-          <t>SOCIEDADES CONTROLADAS</t>
+          <t>OBRAS E INSTALAÇÕES</t>
         </is>
       </c>
       <c r="T20" t="n">
-        <v>11101</v>
+        <v>51000</v>
       </c>
       <c r="U20" t="inlineStr">
         <is>
-          <t>TESOURO ORDINÁRIO - APLICAÇÃO LIVRE</t>
+          <t>RECURSOS PRÓPRIOS</t>
         </is>
       </c>
       <c r="V20" t="inlineStr">
         <is>
-          <t>MANUTENÇÃO E ADEQUAÇÃO DA INFRA-ESTRUTURA ADMINISTRATIVA E OPERACIONAL - TRANSPORTES METROPOLITANOS</t>
+          <t>GÁS COMPETITIVO- EXPANSÃO DA REDE DE GÁS NATURAL</t>
         </is>
       </c>
       <c r="W20" t="inlineStr">
         <is>
-          <t>APOIO ÀS POLÍTICAS PÚBLICAS</t>
+          <t>MINAS GERAÇÃO DE VALOR</t>
         </is>
       </c>
     </row>
@@ -2153,83 +2153,83 @@
         <v>2027</v>
       </c>
       <c r="B21" t="n">
-        <v>1220</v>
+        <v>1300</v>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>SECRETARIA DE ESTADO DE DESENVOLVIMENTO ECONÔMICO - MGS</t>
+          <t>SECRETARIA DE ESTADO DE INFRAESTRUTURA, MOBILIDADE E PARCERIA - TREM METROPOLITANO</t>
         </is>
       </c>
       <c r="D21" t="n">
         <v>3</v>
       </c>
       <c r="E21" t="n">
-        <v>5381</v>
+        <v>5261</v>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>MINAS GERAIS ADMINISTRAÇÃO E SERVIÇOS S.A - MGS</t>
+          <t>TREM METROPOLITANO DE BELO HORIZONTE S.A - TREM METROPOLITANO</t>
         </is>
       </c>
       <c r="G21" t="inlineStr"/>
       <c r="H21" t="n">
-        <v>4</v>
+        <v>26</v>
       </c>
       <c r="I21" t="n">
-        <v>122</v>
+        <v>783</v>
       </c>
       <c r="J21" t="n">
-        <v>57</v>
+        <v>705</v>
       </c>
       <c r="K21" t="n">
         <v>8</v>
       </c>
       <c r="L21" t="n">
-        <v>2</v>
+        <v>11</v>
       </c>
       <c r="M21" t="n">
-        <v>8002</v>
+        <v>8011</v>
       </c>
       <c r="N21" t="n">
-        <v>12650330</v>
+        <v>1000</v>
       </c>
       <c r="O21" t="n">
         <v>0</v>
       </c>
       <c r="P21" t="inlineStr">
         <is>
-          <t>INVESTIMENTOS EM ATIVO FIXO PARA PRESTAÇÃO DE SERVIÇO</t>
+          <t>MANUTENÇÃO E ADEQUAÇÃO DA INFRA-ESTRUTURA ADMINISTRATIVA E OPERACIONAL - TRANSPORTES METROPOLITANOS</t>
         </is>
       </c>
       <c r="Q21" t="inlineStr">
         <is>
-          <t>4610 - IMOBILIZAÇÕES</t>
+          <t>4510 - PARTICIPAÇÃO SOCIETÁRIA</t>
         </is>
       </c>
       <c r="R21" t="n">
-        <v>4614</v>
+        <v>4511</v>
       </c>
       <c r="S21" t="inlineStr">
         <is>
-          <t>MÁQUINAS, APARELHOS E EQUIPAMENTOS</t>
+          <t>SOCIEDADES CONTROLADAS</t>
         </is>
       </c>
       <c r="T21" t="n">
-        <v>51000</v>
+        <v>11101</v>
       </c>
       <c r="U21" t="inlineStr">
         <is>
-          <t>RECURSOS PRÓPRIOS</t>
+          <t>TESOURO ORDINÁRIO - APLICAÇÃO LIVRE</t>
         </is>
       </c>
       <c r="V21" t="inlineStr">
         <is>
-          <t>INVESTIMENTOS EM ATIVO FIXO PARA PRESTAÇÃO DE SERVIÇO</t>
+          <t>MANUTENÇÃO E ADEQUAÇÃO DA INFRA-ESTRUTURA ADMINISTRATIVA E OPERACIONAL - TRANSPORTES METROPOLITANOS</t>
         </is>
       </c>
       <c r="W21" t="inlineStr">
         <is>
-          <t>SOLUÇÕES EM SERVIÇOS DE APOIO TÉCNICO-OPERACIONAL</t>
+          <t>APOIO ÀS POLÍTICAS PÚBLICAS</t>
         </is>
       </c>
     </row>
@@ -2276,7 +2276,7 @@
         <v>8002</v>
       </c>
       <c r="N22" t="n">
-        <v>524600</v>
+        <v>12650330</v>
       </c>
       <c r="O22" t="n">
         <v>0</v>
@@ -2292,11 +2292,11 @@
         </is>
       </c>
       <c r="R22" t="n">
-        <v>4615</v>
+        <v>4614</v>
       </c>
       <c r="S22" t="inlineStr">
         <is>
-          <t>MÓVEIS E UTENSÍLIOS</t>
+          <t>MÁQUINAS, APARELHOS E EQUIPAMENTOS</t>
         </is>
       </c>
       <c r="T22" t="n">
@@ -2361,7 +2361,7 @@
         <v>8002</v>
       </c>
       <c r="N23" t="n">
-        <v>1000</v>
+        <v>524600</v>
       </c>
       <c r="O23" t="n">
         <v>0</v>
@@ -2373,23 +2373,23 @@
       </c>
       <c r="Q23" t="inlineStr">
         <is>
-          <t>4810 - OUTRAS APLICAÇÕES</t>
+          <t>4610 - IMOBILIZAÇÕES</t>
         </is>
       </c>
       <c r="R23" t="n">
-        <v>4810</v>
+        <v>4615</v>
       </c>
       <c r="S23" t="inlineStr">
         <is>
-          <t>OUTRAS APLICAÇÕES</t>
+          <t>MÓVEIS E UTENSÍLIOS</t>
         </is>
       </c>
       <c r="T23" t="n">
-        <v>11101</v>
+        <v>51000</v>
       </c>
       <c r="U23" t="inlineStr">
         <is>
-          <t>TESOURO ORDINÁRIO - APLICAÇÃO LIVRE</t>
+          <t>RECURSOS PRÓPRIOS</t>
         </is>
       </c>
       <c r="V23" t="inlineStr">
@@ -2446,7 +2446,7 @@
         <v>8002</v>
       </c>
       <c r="N24" t="n">
-        <v>4842500</v>
+        <v>1000</v>
       </c>
       <c r="O24" t="n">
         <v>0</v>
@@ -2462,19 +2462,19 @@
         </is>
       </c>
       <c r="R24" t="n">
-        <v>4817</v>
+        <v>4810</v>
       </c>
       <c r="S24" t="inlineStr">
         <is>
-          <t>EQUIPAMENTOS E SOFTWARE</t>
+          <t>OUTRAS APLICAÇÕES</t>
         </is>
       </c>
       <c r="T24" t="n">
-        <v>51000</v>
+        <v>11101</v>
       </c>
       <c r="U24" t="inlineStr">
         <is>
-          <t>RECURSOS PRÓPRIOS</t>
+          <t>TESOURO ORDINÁRIO - APLICAÇÃO LIVRE</t>
         </is>
       </c>
       <c r="V24" t="inlineStr">
@@ -2497,61 +2497,61 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>SECRETARIA DE ESTADO DE DESENVOLVIMENTO ECONÔMICO - CEMIG GERAÇÃO E TRANSMISSÃO</t>
+          <t>SECRETARIA DE ESTADO DE DESENVOLVIMENTO ECONÔMICO - MGS</t>
         </is>
       </c>
       <c r="D25" t="n">
         <v>3</v>
       </c>
       <c r="E25" t="n">
-        <v>5391</v>
+        <v>5381</v>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>CEMIG GERAÇÃO E TRANSMISSÃO S.A - CEMIG GERAÇÃO E TRANSMISSÃO</t>
+          <t>MINAS GERAIS ADMINISTRAÇÃO E SERVIÇOS S.A - MGS</t>
         </is>
       </c>
       <c r="G25" t="inlineStr"/>
       <c r="H25" t="n">
-        <v>25</v>
+        <v>4</v>
       </c>
       <c r="I25" t="n">
-        <v>752</v>
+        <v>122</v>
       </c>
       <c r="J25" t="n">
-        <v>92</v>
+        <v>57</v>
       </c>
       <c r="K25" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="L25" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="M25" t="n">
-        <v>3004</v>
+        <v>8002</v>
       </c>
       <c r="N25" t="n">
-        <v>228410975</v>
+        <v>4842500</v>
       </c>
       <c r="O25" t="n">
         <v>0</v>
       </c>
       <c r="P25" t="inlineStr">
         <is>
-          <t>EXPANSÃO DO SISTEMA DE TRANSMISSÃO</t>
+          <t>INVESTIMENTOS EM ATIVO FIXO PARA PRESTAÇÃO DE SERVIÇO</t>
         </is>
       </c>
       <c r="Q25" t="inlineStr">
         <is>
-          <t>4610 - IMOBILIZAÇÕES</t>
+          <t>4810 - OUTRAS APLICAÇÕES</t>
         </is>
       </c>
       <c r="R25" t="n">
-        <v>4613</v>
+        <v>4817</v>
       </c>
       <c r="S25" t="inlineStr">
         <is>
-          <t>OBRAS E INSTALAÇÕES</t>
+          <t>EQUIPAMENTOS E SOFTWARE</t>
         </is>
       </c>
       <c r="T25" t="n">
@@ -2564,12 +2564,12 @@
       </c>
       <c r="V25" t="inlineStr">
         <is>
-          <t>EXPANSÃO DO SISTEMA DE TRANSMISSÃO</t>
+          <t>INVESTIMENTOS EM ATIVO FIXO PARA PRESTAÇÃO DE SERVIÇO</t>
         </is>
       </c>
       <c r="W25" t="inlineStr">
         <is>
-          <t>TRANSMISSÃO DE ENERGIA ELÉTRICA</t>
+          <t>SOLUÇÕES EM SERVIÇOS DE APOIO TÉCNICO-OPERACIONAL</t>
         </is>
       </c>
     </row>
@@ -2610,20 +2610,20 @@
         <v>3</v>
       </c>
       <c r="L26" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="M26" t="n">
-        <v>3005</v>
+        <v>3004</v>
       </c>
       <c r="N26" t="n">
-        <v>426883823</v>
+        <v>228410975</v>
       </c>
       <c r="O26" t="n">
         <v>0</v>
       </c>
       <c r="P26" t="inlineStr">
         <is>
-          <t xml:space="preserve">REFORMAS DE SUBESTAÇÕES E LINHAS DE TRANSMISSÃO </t>
+          <t>EXPANSÃO DO SISTEMA DE TRANSMISSÃO</t>
         </is>
       </c>
       <c r="Q26" t="inlineStr">
@@ -2649,7 +2649,7 @@
       </c>
       <c r="V26" t="inlineStr">
         <is>
-          <t xml:space="preserve">REFORMAS DE SUBESTAÇÕES E LINHAS DE TRANSMISSÃO </t>
+          <t>EXPANSÃO DO SISTEMA DE TRANSMISSÃO</t>
         </is>
       </c>
       <c r="W26" t="inlineStr">
@@ -2695,20 +2695,20 @@
         <v>3</v>
       </c>
       <c r="L27" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="M27" t="n">
-        <v>3006</v>
+        <v>3005</v>
       </c>
       <c r="N27" t="n">
-        <v>32235731</v>
+        <v>426883823</v>
       </c>
       <c r="O27" t="n">
         <v>0</v>
       </c>
       <c r="P27" t="inlineStr">
         <is>
-          <t>MANUTENÇÃO DA INFRAESTRUTURA DA TRANSMISSÃO</t>
+          <t xml:space="preserve">REFORMAS DE SUBESTAÇÕES E LINHAS DE TRANSMISSÃO </t>
         </is>
       </c>
       <c r="Q27" t="inlineStr">
@@ -2717,11 +2717,11 @@
         </is>
       </c>
       <c r="R27" t="n">
-        <v>4614</v>
+        <v>4613</v>
       </c>
       <c r="S27" t="inlineStr">
         <is>
-          <t>MÁQUINAS, APARELHOS E EQUIPAMENTOS</t>
+          <t>OBRAS E INSTALAÇÕES</t>
         </is>
       </c>
       <c r="T27" t="n">
@@ -2734,7 +2734,7 @@
       </c>
       <c r="V27" t="inlineStr">
         <is>
-          <t>MANUTENÇÃO DA INFRAESTRUTURA DA TRANSMISSÃO</t>
+          <t xml:space="preserve">REFORMAS DE SUBESTAÇÕES E LINHAS DE TRANSMISSÃO </t>
         </is>
       </c>
       <c r="W27" t="inlineStr">
@@ -2780,20 +2780,20 @@
         <v>3</v>
       </c>
       <c r="L28" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="M28" t="n">
-        <v>3009</v>
+        <v>3006</v>
       </c>
       <c r="N28" t="n">
-        <v>56493213</v>
+        <v>32235731</v>
       </c>
       <c r="O28" t="n">
         <v>0</v>
       </c>
       <c r="P28" t="inlineStr">
         <is>
-          <t xml:space="preserve">INVESTIMENTOS PARTICIPAÇÕES SOCIETÁRIAS DA TRANSMISSÃO </t>
+          <t>MANUTENÇÃO DA INFRAESTRUTURA DA TRANSMISSÃO</t>
         </is>
       </c>
       <c r="Q28" t="inlineStr">
@@ -2819,7 +2819,7 @@
       </c>
       <c r="V28" t="inlineStr">
         <is>
-          <t xml:space="preserve">INVESTIMENTOS PARTICIPAÇÕES SOCIETÁRIAS DA TRANSMISSÃO </t>
+          <t>MANUTENÇÃO DA INFRAESTRUTURA DA TRANSMISSÃO</t>
         </is>
       </c>
       <c r="W28" t="inlineStr">
@@ -2859,26 +2859,26 @@
         <v>752</v>
       </c>
       <c r="J29" t="n">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="K29" t="n">
         <v>3</v>
       </c>
       <c r="L29" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="M29" t="n">
-        <v>3001</v>
+        <v>3009</v>
       </c>
       <c r="N29" t="n">
-        <v>1000</v>
+        <v>56493213</v>
       </c>
       <c r="O29" t="n">
         <v>0</v>
       </c>
       <c r="P29" t="inlineStr">
         <is>
-          <t>EXPANSÃO DO SISTEMA DE GERAÇÃO</t>
+          <t xml:space="preserve">INVESTIMENTOS PARTICIPAÇÕES SOCIETÁRIAS DA TRANSMISSÃO </t>
         </is>
       </c>
       <c r="Q29" t="inlineStr">
@@ -2887,11 +2887,11 @@
         </is>
       </c>
       <c r="R29" t="n">
-        <v>4613</v>
+        <v>4614</v>
       </c>
       <c r="S29" t="inlineStr">
         <is>
-          <t>OBRAS E INSTALAÇÕES</t>
+          <t>MÁQUINAS, APARELHOS E EQUIPAMENTOS</t>
         </is>
       </c>
       <c r="T29" t="n">
@@ -2904,12 +2904,12 @@
       </c>
       <c r="V29" t="inlineStr">
         <is>
-          <t>EXPANSÃO DO SISTEMA DE GERAÇÃO</t>
+          <t xml:space="preserve">INVESTIMENTOS PARTICIPAÇÕES SOCIETÁRIAS DA TRANSMISSÃO </t>
         </is>
       </c>
       <c r="W29" t="inlineStr">
         <is>
-          <t xml:space="preserve">GERAÇÃO DE ENERGIA ELÉTRICA </t>
+          <t>TRANSMISSÃO DE ENERGIA ELÉTRICA</t>
         </is>
       </c>
     </row>
@@ -2950,20 +2950,20 @@
         <v>3</v>
       </c>
       <c r="L30" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="M30" t="n">
-        <v>3007</v>
+        <v>3001</v>
       </c>
       <c r="N30" t="n">
-        <v>121588957</v>
+        <v>1000</v>
       </c>
       <c r="O30" t="n">
         <v>0</v>
       </c>
       <c r="P30" t="inlineStr">
         <is>
-          <t xml:space="preserve"> REFORMAS, MELHORIAS E AMPLIAÇÕES DE USINAS</t>
+          <t>EXPANSÃO DO SISTEMA DE GERAÇÃO</t>
         </is>
       </c>
       <c r="Q30" t="inlineStr">
@@ -2972,11 +2972,11 @@
         </is>
       </c>
       <c r="R30" t="n">
-        <v>4614</v>
+        <v>4613</v>
       </c>
       <c r="S30" t="inlineStr">
         <is>
-          <t>MÁQUINAS, APARELHOS E EQUIPAMENTOS</t>
+          <t>OBRAS E INSTALAÇÕES</t>
         </is>
       </c>
       <c r="T30" t="n">
@@ -2989,7 +2989,7 @@
       </c>
       <c r="V30" t="inlineStr">
         <is>
-          <t xml:space="preserve"> REFORMAS, MELHORIAS E AMPLIAÇÕES DE USINAS</t>
+          <t>EXPANSÃO DO SISTEMA DE GERAÇÃO</t>
         </is>
       </c>
       <c r="W30" t="inlineStr">
@@ -3035,20 +3035,20 @@
         <v>3</v>
       </c>
       <c r="L31" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="M31" t="n">
-        <v>3008</v>
+        <v>3007</v>
       </c>
       <c r="N31" t="n">
-        <v>28627843</v>
+        <v>121588957</v>
       </c>
       <c r="O31" t="n">
         <v>0</v>
       </c>
       <c r="P31" t="inlineStr">
         <is>
-          <t>MANUTENÇÃO DA INFRAESTRUTURA DA GERAÇÃO</t>
+          <t xml:space="preserve"> REFORMAS, MELHORIAS E AMPLIAÇÕES DE USINAS</t>
         </is>
       </c>
       <c r="Q31" t="inlineStr">
@@ -3074,7 +3074,7 @@
       </c>
       <c r="V31" t="inlineStr">
         <is>
-          <t>MANUTENÇÃO DA INFRAESTRUTURA DA GERAÇÃO</t>
+          <t xml:space="preserve"> REFORMAS, MELHORIAS E AMPLIAÇÕES DE USINAS</t>
         </is>
       </c>
       <c r="W31" t="inlineStr">
@@ -3120,20 +3120,20 @@
         <v>3</v>
       </c>
       <c r="L32" t="n">
-        <v>14</v>
+        <v>8</v>
       </c>
       <c r="M32" t="n">
-        <v>3014</v>
+        <v>3008</v>
       </c>
       <c r="N32" t="n">
-        <v>1080197578</v>
+        <v>28627843</v>
       </c>
       <c r="O32" t="n">
         <v>0</v>
       </c>
       <c r="P32" t="inlineStr">
         <is>
-          <t>INVESTIMENTOS EM PARTICIPAÇÕES SOCIETÁRIAS DA GERAÇÃO</t>
+          <t>MANUTENÇÃO DA INFRAESTRUTURA DA GERAÇÃO</t>
         </is>
       </c>
       <c r="Q32" t="inlineStr">
@@ -3159,7 +3159,7 @@
       </c>
       <c r="V32" t="inlineStr">
         <is>
-          <t>INVESTIMENTOS EM PARTICIPAÇÕES SOCIETÁRIAS DA GERAÇÃO</t>
+          <t>MANUTENÇÃO DA INFRAESTRUTURA DA GERAÇÃO</t>
         </is>
       </c>
       <c r="W32" t="inlineStr">
@@ -3177,18 +3177,18 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>SECRETARIA DE ESTADO DE DESENVOLVIMENTO ECONÔMICO - CEMIG DISTRIBUIDORA</t>
+          <t>SECRETARIA DE ESTADO DE DESENVOLVIMENTO ECONÔMICO - CEMIG GERAÇÃO E TRANSMISSÃO</t>
         </is>
       </c>
       <c r="D33" t="n">
         <v>3</v>
       </c>
       <c r="E33" t="n">
-        <v>5401</v>
+        <v>5391</v>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>CEMIG DISTRIBUIÇÃO S.A - CEMIG DISTRIBUIDORA</t>
+          <t>CEMIG GERAÇÃO E TRANSMISSÃO S.A - CEMIG GERAÇÃO E TRANSMISSÃO</t>
         </is>
       </c>
       <c r="G33" t="inlineStr"/>
@@ -3199,26 +3199,26 @@
         <v>752</v>
       </c>
       <c r="J33" t="n">
-        <v>72</v>
+        <v>94</v>
       </c>
       <c r="K33" t="n">
         <v>3</v>
       </c>
       <c r="L33" t="n">
-        <v>2</v>
+        <v>14</v>
       </c>
       <c r="M33" t="n">
-        <v>3002</v>
+        <v>3014</v>
       </c>
       <c r="N33" t="n">
-        <v>5320034427</v>
+        <v>1080197578</v>
       </c>
       <c r="O33" t="n">
         <v>0</v>
       </c>
       <c r="P33" t="inlineStr">
         <is>
-          <t xml:space="preserve">EXECUÇÃO DO PLANO DE DESENVOLVIMENTO DA DISTRIBUIDORA (PDD) </t>
+          <t>INVESTIMENTOS EM PARTICIPAÇÕES SOCIETÁRIAS DA GERAÇÃO</t>
         </is>
       </c>
       <c r="Q33" t="inlineStr">
@@ -3244,12 +3244,12 @@
       </c>
       <c r="V33" t="inlineStr">
         <is>
-          <t xml:space="preserve">EXECUÇÃO DO PLANO DE DESENVOLVIMENTO DA DISTRIBUIDORA (PDD) </t>
+          <t>INVESTIMENTOS EM PARTICIPAÇÕES SOCIETÁRIAS DA GERAÇÃO</t>
         </is>
       </c>
       <c r="W33" t="inlineStr">
         <is>
-          <t>DISTRIBUIÇÃO DE ENERGIA ELÉTRICA</t>
+          <t xml:space="preserve">GERAÇÃO DE ENERGIA ELÉTRICA </t>
         </is>
       </c>
     </row>
@@ -3290,20 +3290,20 @@
         <v>3</v>
       </c>
       <c r="L34" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="M34" t="n">
-        <v>3003</v>
+        <v>3002</v>
       </c>
       <c r="N34" t="n">
-        <v>250370467</v>
+        <v>5320034427</v>
       </c>
       <c r="O34" t="n">
         <v>0</v>
       </c>
       <c r="P34" t="inlineStr">
         <is>
-          <t xml:space="preserve">MANUTENÇÃO DA INFRAESTRUTURA DA DISTRIBUIÇÃO </t>
+          <t xml:space="preserve">EXECUÇÃO DO PLANO DE DESENVOLVIMENTO DA DISTRIBUIDORA (PDD) </t>
         </is>
       </c>
       <c r="Q34" t="inlineStr">
@@ -3329,10 +3329,95 @@
       </c>
       <c r="V34" t="inlineStr">
         <is>
+          <t xml:space="preserve">EXECUÇÃO DO PLANO DE DESENVOLVIMENTO DA DISTRIBUIDORA (PDD) </t>
+        </is>
+      </c>
+      <c r="W34" t="inlineStr">
+        <is>
+          <t>DISTRIBUIÇÃO DE ENERGIA ELÉTRICA</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="n">
+        <v>2027</v>
+      </c>
+      <c r="B35" t="n">
+        <v>1220</v>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>SECRETARIA DE ESTADO DE DESENVOLVIMENTO ECONÔMICO - CEMIG DISTRIBUIDORA</t>
+        </is>
+      </c>
+      <c r="D35" t="n">
+        <v>3</v>
+      </c>
+      <c r="E35" t="n">
+        <v>5401</v>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>CEMIG DISTRIBUIÇÃO S.A - CEMIG DISTRIBUIDORA</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr"/>
+      <c r="H35" t="n">
+        <v>25</v>
+      </c>
+      <c r="I35" t="n">
+        <v>752</v>
+      </c>
+      <c r="J35" t="n">
+        <v>72</v>
+      </c>
+      <c r="K35" t="n">
+        <v>3</v>
+      </c>
+      <c r="L35" t="n">
+        <v>3</v>
+      </c>
+      <c r="M35" t="n">
+        <v>3003</v>
+      </c>
+      <c r="N35" t="n">
+        <v>250370467</v>
+      </c>
+      <c r="O35" t="n">
+        <v>0</v>
+      </c>
+      <c r="P35" t="inlineStr">
+        <is>
           <t xml:space="preserve">MANUTENÇÃO DA INFRAESTRUTURA DA DISTRIBUIÇÃO </t>
         </is>
       </c>
-      <c r="W34" t="inlineStr">
+      <c r="Q35" t="inlineStr">
+        <is>
+          <t>4610 - IMOBILIZAÇÕES</t>
+        </is>
+      </c>
+      <c r="R35" t="n">
+        <v>4614</v>
+      </c>
+      <c r="S35" t="inlineStr">
+        <is>
+          <t>MÁQUINAS, APARELHOS E EQUIPAMENTOS</t>
+        </is>
+      </c>
+      <c r="T35" t="n">
+        <v>51000</v>
+      </c>
+      <c r="U35" t="inlineStr">
+        <is>
+          <t>RECURSOS PRÓPRIOS</t>
+        </is>
+      </c>
+      <c r="V35" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MANUTENÇÃO DA INFRAESTRUTURA DA DISTRIBUIÇÃO </t>
+        </is>
+      </c>
+      <c r="W35" t="inlineStr">
         <is>
           <t>DISTRIBUIÇÃO DE ENERGIA ELÉTRICA</t>
         </is>

</xml_diff>